<commit_message>
Relabel caffeine column as "unit not stated" and rebuild Phase 1 outputs
The dataset does not document what unit the caffeine column is measured in,
and the source page could not be reached to confirm it. The label previously
implied cups per day, which was an assumption rather than a fact.

Both notebooks and both reports were re-run after the change so the label is
consistent everywhere it appears.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/visualize/report.xlsx
+++ b/visualize/report.xlsx
@@ -5250,7 +5250,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Caffeine (cups/day)</t>
+          <t>Caffeine intake (per day, unit not stated)</t>
         </is>
       </c>
       <c r="B55" s="41" t="n">
@@ -7201,7 +7201,7 @@
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>Caffeine (cups/day)</t>
+          <t>Caffeine intake (per day, unit not stated)</t>
         </is>
       </c>
       <c r="B135" s="41" t="n">

</xml_diff>